<commit_message>
Team Principal: contract negotiation, dismissed engineers, drivers panel
Hiring now opens a contract dialog: the engineer's offer (target length and
salary in half-coin steps) with a live reaction hint, a refusal costing
confidence and closing him until season end, per spec section 8.3. Eligibility
stays trust OR prestige. A dismissed engineer stays first in the market but
won't return to that team this season, then asks a premium. The local offer
is only open before the first race. Drivers (2 + reserve placeholder) are
shown with the same card model as engineers, and the header and tab bar are
now one sticky container. Engineer value is no longer displayed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/engineers_db.xlsx
+++ b/data/source/engineers_db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76929c7f1b9de68b/Documents/Dada/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_40D776E31060002FED7EA0345B012E3F6DCBECF1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8602AB84-D492-44F5-B22B-47F81F005001}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="11_40D776E31060002FED7EA0345B012E3F6DCBECF1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{927B6409-4025-48CF-B081-9115D06AE9BF}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="450" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -2133,6 +2133,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2633,7 +2637,7 @@
         <v>24</v>
       </c>
       <c r="D5">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -2674,7 +2678,7 @@
         <v>14</v>
       </c>
       <c r="D6">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E6" t="s">
         <v>15</v>
@@ -2715,7 +2719,7 @@
         <v>19</v>
       </c>
       <c r="D7">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
@@ -2756,7 +2760,7 @@
         <v>21</v>
       </c>
       <c r="D8">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E8" t="s">
         <v>15</v>
@@ -2812,7 +2816,7 @@
         <v>7</v>
       </c>
       <c r="I9">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
         <v>25</v>
@@ -2838,7 +2842,7 @@
         <v>14</v>
       </c>
       <c r="D10">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E10" t="s">
         <v>15</v>
@@ -2853,7 +2857,7 @@
         <v>7</v>
       </c>
       <c r="I10">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J10" t="s">
         <v>16</v>
@@ -2879,7 +2883,7 @@
         <v>19</v>
       </c>
       <c r="D11">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E11" t="s">
         <v>15</v>
@@ -2920,7 +2924,7 @@
         <v>21</v>
       </c>
       <c r="D12">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E12" t="s">
         <v>15</v>
@@ -2961,7 +2965,7 @@
         <v>24</v>
       </c>
       <c r="D13">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E13" t="s">
         <v>15</v>
@@ -3002,7 +3006,7 @@
         <v>14</v>
       </c>
       <c r="D14">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
         <v>15</v>
@@ -3043,7 +3047,7 @@
         <v>19</v>
       </c>
       <c r="D15">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
         <v>15</v>
@@ -3058,7 +3062,7 @@
         <v>7</v>
       </c>
       <c r="I15">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J15" t="s">
         <v>16</v>
@@ -3084,7 +3088,7 @@
         <v>21</v>
       </c>
       <c r="D16">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E16" t="s">
         <v>15</v>
@@ -3125,7 +3129,7 @@
         <v>24</v>
       </c>
       <c r="D17">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
         <v>15</v>
@@ -3166,7 +3170,7 @@
         <v>14</v>
       </c>
       <c r="D18">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
@@ -3181,7 +3185,7 @@
         <v>7</v>
       </c>
       <c r="I18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J18" t="s">
         <v>43</v>
@@ -3248,7 +3252,7 @@
         <v>21</v>
       </c>
       <c r="D20">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E20" t="s">
         <v>15</v>
@@ -3263,7 +3267,7 @@
         <v>7</v>
       </c>
       <c r="I20">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J20" t="s">
         <v>25</v>
@@ -3289,7 +3293,7 @@
         <v>24</v>
       </c>
       <c r="D21">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
@@ -3304,7 +3308,7 @@
         <v>7</v>
       </c>
       <c r="I21">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J21" t="s">
         <v>16</v>
@@ -3345,7 +3349,7 @@
         <v>7</v>
       </c>
       <c r="I22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J22" t="s">
         <v>30</v>
@@ -3386,7 +3390,7 @@
         <v>7</v>
       </c>
       <c r="I23">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J23" t="s">
         <v>16</v>
@@ -3453,7 +3457,7 @@
         <v>24</v>
       </c>
       <c r="D25">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E25" t="s">
         <v>15</v>
@@ -3494,7 +3498,7 @@
         <v>14</v>
       </c>
       <c r="D26">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E26" t="s">
         <v>15</v>
@@ -3509,7 +3513,7 @@
         <v>7</v>
       </c>
       <c r="I26">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J26" t="s">
         <v>16</v>
@@ -3535,7 +3539,7 @@
         <v>19</v>
       </c>
       <c r="D27">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E27" t="s">
         <v>15</v>
@@ -3550,7 +3554,7 @@
         <v>7</v>
       </c>
       <c r="I27">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J27" t="s">
         <v>16</v>
@@ -3617,7 +3621,7 @@
         <v>24</v>
       </c>
       <c r="D29">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E29" t="s">
         <v>15</v>
@@ -3632,7 +3636,7 @@
         <v>7</v>
       </c>
       <c r="I29">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J29" t="s">
         <v>16</v>
@@ -3658,7 +3662,7 @@
         <v>19</v>
       </c>
       <c r="D30">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E30" t="s">
         <v>15</v>
@@ -3673,7 +3677,7 @@
         <v>7</v>
       </c>
       <c r="I30">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J30" t="s">
         <v>25</v>
@@ -3699,7 +3703,7 @@
         <v>21</v>
       </c>
       <c r="D31">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E31" t="s">
         <v>15</v>
@@ -3714,7 +3718,7 @@
         <v>7</v>
       </c>
       <c r="I31">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J31" t="s">
         <v>25</v>
@@ -3781,7 +3785,7 @@
         <v>14</v>
       </c>
       <c r="D33">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E33" t="s">
         <v>15</v>
@@ -3822,7 +3826,7 @@
         <v>19</v>
       </c>
       <c r="D34">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E34" t="s">
         <v>15</v>
@@ -3863,7 +3867,7 @@
         <v>21</v>
       </c>
       <c r="D35">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E35" t="s">
         <v>15</v>
@@ -3878,7 +3882,7 @@
         <v>7</v>
       </c>
       <c r="I35">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J35" t="s">
         <v>16</v>
@@ -3919,7 +3923,7 @@
         <v>7</v>
       </c>
       <c r="I36">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J36" t="s">
         <v>30</v>
@@ -3945,7 +3949,7 @@
         <v>14</v>
       </c>
       <c r="D37">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E37" t="s">
         <v>15</v>
@@ -3960,7 +3964,7 @@
         <v>7</v>
       </c>
       <c r="I37">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J37" t="s">
         <v>16</v>
@@ -3986,7 +3990,7 @@
         <v>19</v>
       </c>
       <c r="D38">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E38" t="s">
         <v>15</v>
@@ -4001,7 +4005,7 @@
         <v>7</v>
       </c>
       <c r="I38">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J38" t="s">
         <v>16</v>
@@ -4027,7 +4031,7 @@
         <v>21</v>
       </c>
       <c r="D39">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E39" t="s">
         <v>15</v>
@@ -4042,7 +4046,7 @@
         <v>7</v>
       </c>
       <c r="I39">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J39" t="s">
         <v>16</v>
@@ -4068,7 +4072,7 @@
         <v>24</v>
       </c>
       <c r="D40">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E40" t="s">
         <v>15</v>
@@ -4083,7 +4087,7 @@
         <v>7</v>
       </c>
       <c r="I40">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J40" t="s">
         <v>16</v>
@@ -4124,7 +4128,7 @@
         <v>7</v>
       </c>
       <c r="I41">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J41" t="s">
         <v>75</v>
@@ -4165,7 +4169,7 @@
         <v>7</v>
       </c>
       <c r="I42">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J42" t="s">
         <v>16</v>
@@ -4206,7 +4210,7 @@
         <v>7</v>
       </c>
       <c r="I43">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J43" t="s">
         <v>16</v>
@@ -4247,7 +4251,7 @@
         <v>7</v>
       </c>
       <c r="I44">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J44" t="s">
         <v>16</v>
@@ -4288,7 +4292,7 @@
         <v>7</v>
       </c>
       <c r="I45">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
         <v>75</v>
@@ -4568,7 +4572,7 @@
         <v>3</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J53" t="s">
         <v>25</v>
@@ -4638,7 +4642,7 @@
         <v>3</v>
       </c>
       <c r="I55">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J55" t="s">
         <v>16</v>
@@ -4673,7 +4677,7 @@
         <v>3</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J56" t="s">
         <v>98</v>
@@ -4708,7 +4712,7 @@
         <v>3</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J57" t="s">
         <v>16</v>
@@ -4848,7 +4852,7 @@
         <v>3</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J61" t="s">
         <v>104</v>
@@ -4918,7 +4922,7 @@
         <v>3</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J63" t="s">
         <v>98</v>
@@ -5023,7 +5027,7 @@
         <v>3</v>
       </c>
       <c r="I66">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J66" t="s">
         <v>25</v>
@@ -5163,7 +5167,7 @@
         <v>7</v>
       </c>
       <c r="I70">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J70" t="s">
         <v>16</v>
@@ -5268,7 +5272,7 @@
         <v>3</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J73" t="s">
         <v>25</v>
@@ -5443,7 +5447,7 @@
         <v>3</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J78" t="s">
         <v>30</v>
@@ -5583,7 +5587,7 @@
         <v>7</v>
       </c>
       <c r="I82">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J82" t="s">
         <v>30</v>
@@ -5793,7 +5797,7 @@
         <v>3</v>
       </c>
       <c r="I88">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J88" t="s">
         <v>141</v>
@@ -5898,7 +5902,7 @@
         <v>3</v>
       </c>
       <c r="I91">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J91" t="s">
         <v>146</v>
@@ -6038,7 +6042,7 @@
         <v>7</v>
       </c>
       <c r="I95">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J95" t="s">
         <v>75</v>
@@ -6143,7 +6147,7 @@
         <v>3</v>
       </c>
       <c r="I98">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J98" t="s">
         <v>25</v>
@@ -6178,7 +6182,7 @@
         <v>3</v>
       </c>
       <c r="I99">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J99" t="s">
         <v>155</v>
@@ -6248,7 +6252,7 @@
         <v>3</v>
       </c>
       <c r="I101">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J101" t="s">
         <v>98</v>
@@ -6353,7 +6357,7 @@
         <v>3</v>
       </c>
       <c r="I104">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J104" t="s">
         <v>30</v>
@@ -6458,7 +6462,7 @@
         <v>7</v>
       </c>
       <c r="I107">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J107" t="s">
         <v>25</v>
@@ -6528,7 +6532,7 @@
         <v>3</v>
       </c>
       <c r="I109">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J109" t="s">
         <v>16</v>
@@ -6598,7 +6602,7 @@
         <v>3</v>
       </c>
       <c r="I111">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J111" t="s">
         <v>16</v>
@@ -6633,7 +6637,7 @@
         <v>3</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J112" t="s">
         <v>64</v>
@@ -6668,7 +6672,7 @@
         <v>3</v>
       </c>
       <c r="I113">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J113" t="s">
         <v>64</v>
@@ -6843,7 +6847,7 @@
         <v>7</v>
       </c>
       <c r="I118">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J118" t="s">
         <v>16</v>
@@ -7263,7 +7267,7 @@
         <v>3</v>
       </c>
       <c r="I130">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J130" t="s">
         <v>25</v>
@@ -7403,7 +7407,7 @@
         <v>3</v>
       </c>
       <c r="I134">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J134" t="s">
         <v>64</v>
@@ -7438,7 +7442,7 @@
         <v>3</v>
       </c>
       <c r="I135">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J135" t="s">
         <v>198</v>
@@ -7473,7 +7477,7 @@
         <v>3</v>
       </c>
       <c r="I136">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J136" t="s">
         <v>25</v>
@@ -7508,7 +7512,7 @@
         <v>7</v>
       </c>
       <c r="I137">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J137" t="s">
         <v>201</v>
@@ -7648,7 +7652,7 @@
         <v>3</v>
       </c>
       <c r="I141">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J141" t="s">
         <v>207</v>
@@ -7753,7 +7757,7 @@
         <v>3</v>
       </c>
       <c r="I144">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J144" t="s">
         <v>211</v>
@@ -7788,7 +7792,7 @@
         <v>3</v>
       </c>
       <c r="I145">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J145" t="s">
         <v>213</v>
@@ -7963,7 +7967,7 @@
         <v>3</v>
       </c>
       <c r="I150">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J150" t="s">
         <v>16</v>
@@ -8033,7 +8037,7 @@
         <v>7</v>
       </c>
       <c r="I152">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J152" t="s">
         <v>25</v>
@@ -8103,7 +8107,7 @@
         <v>3</v>
       </c>
       <c r="I154">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J154" t="s">
         <v>30</v>
@@ -8138,7 +8142,7 @@
         <v>3</v>
       </c>
       <c r="I155">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J155" t="s">
         <v>30</v>
@@ -8173,7 +8177,7 @@
         <v>7</v>
       </c>
       <c r="I156">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J156" t="s">
         <v>64</v>
@@ -8278,7 +8282,7 @@
         <v>3</v>
       </c>
       <c r="I159">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J159" t="s">
         <v>184</v>
@@ -8313,7 +8317,7 @@
         <v>3</v>
       </c>
       <c r="I160">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J160" t="s">
         <v>25</v>
@@ -8348,7 +8352,7 @@
         <v>7</v>
       </c>
       <c r="I161">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J161" t="s">
         <v>64</v>
@@ -8453,7 +8457,7 @@
         <v>3</v>
       </c>
       <c r="I164">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J164" t="s">
         <v>16</v>
@@ -8593,7 +8597,7 @@
         <v>3</v>
       </c>
       <c r="I168">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J168" t="s">
         <v>25</v>
@@ -8663,7 +8667,7 @@
         <v>3</v>
       </c>
       <c r="I170">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J170" t="s">
         <v>16</v>
@@ -8768,7 +8772,7 @@
         <v>3</v>
       </c>
       <c r="I173">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J173" t="s">
         <v>16</v>
@@ -8803,7 +8807,7 @@
         <v>3</v>
       </c>
       <c r="I174">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J174" t="s">
         <v>16</v>
@@ -8838,7 +8842,7 @@
         <v>3</v>
       </c>
       <c r="I175">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J175" t="s">
         <v>64</v>
@@ -8873,7 +8877,7 @@
         <v>3</v>
       </c>
       <c r="I176">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J176" t="s">
         <v>25</v>
@@ -8908,7 +8912,7 @@
         <v>7</v>
       </c>
       <c r="I177">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J177" t="s">
         <v>16</v>
@@ -9013,7 +9017,7 @@
         <v>3</v>
       </c>
       <c r="I180">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J180" t="s">
         <v>25</v>
@@ -9048,7 +9052,7 @@
         <v>3</v>
       </c>
       <c r="I181">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J181" t="s">
         <v>25</v>
@@ -9118,7 +9122,7 @@
         <v>3</v>
       </c>
       <c r="I183">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J183" t="s">
         <v>260</v>
@@ -9153,7 +9157,7 @@
         <v>3</v>
       </c>
       <c r="I184">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J184" t="s">
         <v>136</v>
@@ -9293,7 +9297,7 @@
         <v>3</v>
       </c>
       <c r="I188">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J188" t="s">
         <v>108</v>
@@ -9363,7 +9367,7 @@
         <v>3</v>
       </c>
       <c r="I190">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J190" t="s">
         <v>270</v>
@@ -9433,7 +9437,7 @@
         <v>3</v>
       </c>
       <c r="I192">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J192" t="s">
         <v>30</v>
@@ -9538,7 +9542,7 @@
         <v>3</v>
       </c>
       <c r="I195">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J195" t="s">
         <v>184</v>
@@ -9643,7 +9647,7 @@
         <v>3</v>
       </c>
       <c r="I198">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J198" t="s">
         <v>30</v>
@@ -9713,7 +9717,7 @@
         <v>3</v>
       </c>
       <c r="I200">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J200" t="s">
         <v>75</v>
@@ -9748,7 +9752,7 @@
         <v>3</v>
       </c>
       <c r="I201">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J201" t="s">
         <v>16</v>
@@ -9783,7 +9787,7 @@
         <v>3</v>
       </c>
       <c r="I202">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J202" t="s">
         <v>16</v>
@@ -9923,7 +9927,7 @@
         <v>3</v>
       </c>
       <c r="I206">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J206" t="s">
         <v>131</v>
@@ -9993,7 +9997,7 @@
         <v>3</v>
       </c>
       <c r="I208">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J208" t="s">
         <v>25</v>
@@ -10063,7 +10067,7 @@
         <v>3</v>
       </c>
       <c r="I210">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J210" t="s">
         <v>160</v>
@@ -10168,7 +10172,7 @@
         <v>3</v>
       </c>
       <c r="I213">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J213" t="s">
         <v>131</v>
@@ -10273,7 +10277,7 @@
         <v>3</v>
       </c>
       <c r="I216">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J216" t="s">
         <v>88</v>
@@ -10378,7 +10382,7 @@
         <v>3</v>
       </c>
       <c r="I219">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J219" t="s">
         <v>303</v>
@@ -10483,7 +10487,7 @@
         <v>3</v>
       </c>
       <c r="I222">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J222" t="s">
         <v>146</v>
@@ -10623,7 +10627,7 @@
         <v>7</v>
       </c>
       <c r="I226">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J226" t="s">
         <v>16</v>
@@ -10658,7 +10662,7 @@
         <v>3</v>
       </c>
       <c r="I227">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J227" t="s">
         <v>98</v>
@@ -10693,7 +10697,7 @@
         <v>3</v>
       </c>
       <c r="I228">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J228" t="s">
         <v>16</v>
@@ -10763,7 +10767,7 @@
         <v>3</v>
       </c>
       <c r="I230">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J230" t="s">
         <v>75</v>
@@ -11008,7 +11012,7 @@
         <v>7</v>
       </c>
       <c r="I237">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J237" t="s">
         <v>16</v>
@@ -11113,7 +11117,7 @@
         <v>3</v>
       </c>
       <c r="I240">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J240" t="s">
         <v>227</v>
@@ -11393,7 +11397,7 @@
         <v>3</v>
       </c>
       <c r="I248">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J248" t="s">
         <v>25</v>
@@ -11463,7 +11467,7 @@
         <v>3</v>
       </c>
       <c r="I250">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J250" t="s">
         <v>64</v>
@@ -11498,7 +11502,7 @@
         <v>3</v>
       </c>
       <c r="I251">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J251" t="s">
         <v>75</v>
@@ -11533,7 +11537,7 @@
         <v>3</v>
       </c>
       <c r="I252">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J252" t="s">
         <v>342</v>
@@ -11673,7 +11677,7 @@
         <v>3</v>
       </c>
       <c r="I256">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J256" t="s">
         <v>342</v>
@@ -11813,7 +11817,7 @@
         <v>3</v>
       </c>
       <c r="I260">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J260" t="s">
         <v>264</v>
@@ -11848,7 +11852,7 @@
         <v>3</v>
       </c>
       <c r="I261">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J261" t="s">
         <v>25</v>
@@ -11883,7 +11887,7 @@
         <v>3</v>
       </c>
       <c r="I262">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J262" t="s">
         <v>25</v>
@@ -12128,7 +12132,7 @@
         <v>3</v>
       </c>
       <c r="I269">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J269" t="s">
         <v>64</v>
@@ -12198,7 +12202,7 @@
         <v>7</v>
       </c>
       <c r="I271">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J271" t="s">
         <v>16</v>
@@ -12268,7 +12272,7 @@
         <v>3</v>
       </c>
       <c r="I273">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J273" t="s">
         <v>367</v>
@@ -12303,7 +12307,7 @@
         <v>3</v>
       </c>
       <c r="I274">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J274" t="s">
         <v>157</v>
@@ -12338,7 +12342,7 @@
         <v>3</v>
       </c>
       <c r="I275">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J275" t="s">
         <v>115</v>
@@ -12373,7 +12377,7 @@
         <v>3</v>
       </c>
       <c r="I276">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J276" t="s">
         <v>246</v>
@@ -12478,7 +12482,7 @@
         <v>3</v>
       </c>
       <c r="I279">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J279" t="s">
         <v>16</v>
@@ -12548,7 +12552,7 @@
         <v>3</v>
       </c>
       <c r="I281">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J281" t="s">
         <v>64</v>
@@ -12723,7 +12727,7 @@
         <v>3</v>
       </c>
       <c r="I286">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J286" t="s">
         <v>16</v>
@@ -12793,7 +12797,7 @@
         <v>3</v>
       </c>
       <c r="I288">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J288" t="s">
         <v>30</v>
@@ -13038,7 +13042,7 @@
         <v>7</v>
       </c>
       <c r="I295">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J295" t="s">
         <v>108</v>
@@ -13108,7 +13112,7 @@
         <v>3</v>
       </c>
       <c r="I297">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J297" t="s">
         <v>25</v>
@@ -13143,7 +13147,7 @@
         <v>3</v>
       </c>
       <c r="I298">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J298" t="s">
         <v>395</v>
@@ -13213,7 +13217,7 @@
         <v>7</v>
       </c>
       <c r="I300">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J300" t="s">
         <v>16</v>
@@ -13283,7 +13287,7 @@
         <v>7</v>
       </c>
       <c r="I302">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J302" t="s">
         <v>16</v>
@@ -13318,7 +13322,7 @@
         <v>3</v>
       </c>
       <c r="I303">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J303" t="s">
         <v>16</v>
@@ -13458,7 +13462,7 @@
         <v>3</v>
       </c>
       <c r="I307">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J307" t="s">
         <v>64</v>
@@ -13633,7 +13637,7 @@
         <v>3</v>
       </c>
       <c r="I312">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J312" t="s">
         <v>160</v>
@@ -13668,7 +13672,7 @@
         <v>3</v>
       </c>
       <c r="I313">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J313" t="s">
         <v>248</v>
@@ -13808,7 +13812,7 @@
         <v>3</v>
       </c>
       <c r="I317">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J317" t="s">
         <v>415</v>
@@ -13948,7 +13952,7 @@
         <v>3</v>
       </c>
       <c r="I321">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J321" t="s">
         <v>64</v>
@@ -14088,7 +14092,7 @@
         <v>3</v>
       </c>
       <c r="I325">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J325" t="s">
         <v>16</v>
@@ -14123,7 +14127,7 @@
         <v>7</v>
       </c>
       <c r="I326">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J326" t="s">
         <v>16</v>
@@ -14298,7 +14302,7 @@
         <v>3</v>
       </c>
       <c r="I331">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J331" t="s">
         <v>395</v>
@@ -14403,7 +14407,7 @@
         <v>3</v>
       </c>
       <c r="I334">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J334" t="s">
         <v>160</v>
@@ -14438,7 +14442,7 @@
         <v>3</v>
       </c>
       <c r="I335">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J335" t="s">
         <v>435</v>
@@ -14473,7 +14477,7 @@
         <v>3</v>
       </c>
       <c r="I336">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J336" t="s">
         <v>136</v>
@@ -14508,7 +14512,7 @@
         <v>3</v>
       </c>
       <c r="I337">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J337" t="s">
         <v>16</v>
@@ -14543,7 +14547,7 @@
         <v>3</v>
       </c>
       <c r="I338">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J338" t="s">
         <v>439</v>
@@ -14753,7 +14757,7 @@
         <v>3</v>
       </c>
       <c r="I344">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J344" t="s">
         <v>108</v>
@@ -14823,7 +14827,7 @@
         <v>3</v>
       </c>
       <c r="I346">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J346" t="s">
         <v>98</v>
@@ -14893,7 +14897,7 @@
         <v>3</v>
       </c>
       <c r="I348">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J348" t="s">
         <v>16</v>
@@ -14963,7 +14967,7 @@
         <v>3</v>
       </c>
       <c r="I350">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J350" t="s">
         <v>25</v>
@@ -14998,7 +15002,7 @@
         <v>3</v>
       </c>
       <c r="I351">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J351" t="s">
         <v>455</v>
@@ -15103,7 +15107,7 @@
         <v>3</v>
       </c>
       <c r="I354">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J354" t="s">
         <v>16</v>
@@ -15138,7 +15142,7 @@
         <v>3</v>
       </c>
       <c r="I355">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J355" t="s">
         <v>64</v>
@@ -15243,7 +15247,7 @@
         <v>7</v>
       </c>
       <c r="I358">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J358" t="s">
         <v>136</v>
@@ -15278,7 +15282,7 @@
         <v>3</v>
       </c>
       <c r="I359">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J359" t="s">
         <v>466</v>
@@ -15383,7 +15387,7 @@
         <v>3</v>
       </c>
       <c r="I362">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J362" t="s">
         <v>25</v>
@@ -15558,7 +15562,7 @@
         <v>3</v>
       </c>
       <c r="I367">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J367" t="s">
         <v>476</v>
@@ -15593,7 +15597,7 @@
         <v>3</v>
       </c>
       <c r="I368">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J368" t="s">
         <v>64</v>
@@ -15978,7 +15982,7 @@
         <v>3</v>
       </c>
       <c r="I379">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J379" t="s">
         <v>180</v>
@@ -16013,7 +16017,7 @@
         <v>7</v>
       </c>
       <c r="I380">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J380" t="s">
         <v>30</v>
@@ -16083,7 +16087,7 @@
         <v>3</v>
       </c>
       <c r="I382">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J382" t="s">
         <v>494</v>
@@ -16118,7 +16122,7 @@
         <v>3</v>
       </c>
       <c r="I383">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J383" t="s">
         <v>25</v>
@@ -16258,7 +16262,7 @@
         <v>3</v>
       </c>
       <c r="I387">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J387" t="s">
         <v>270</v>
@@ -16363,7 +16367,7 @@
         <v>3</v>
       </c>
       <c r="I390">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J390" t="s">
         <v>25</v>
@@ -16398,7 +16402,7 @@
         <v>3</v>
       </c>
       <c r="I391">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J391" t="s">
         <v>338</v>
@@ -16468,7 +16472,7 @@
         <v>3</v>
       </c>
       <c r="I393">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J393" t="s">
         <v>16</v>
@@ -16503,7 +16507,7 @@
         <v>3</v>
       </c>
       <c r="I394">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J394" t="s">
         <v>25</v>
@@ -16538,7 +16542,7 @@
         <v>3</v>
       </c>
       <c r="I395">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J395" t="s">
         <v>16</v>
@@ -16573,7 +16577,7 @@
         <v>3</v>
       </c>
       <c r="I396">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J396" t="s">
         <v>16</v>
@@ -16608,7 +16612,7 @@
         <v>3</v>
       </c>
       <c r="I397">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J397" t="s">
         <v>30</v>
@@ -16678,7 +16682,7 @@
         <v>3</v>
       </c>
       <c r="I399">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J399" t="s">
         <v>30</v>
@@ -16713,7 +16717,7 @@
         <v>3</v>
       </c>
       <c r="I400">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J400" t="s">
         <v>264</v>
@@ -16748,7 +16752,7 @@
         <v>3</v>
       </c>
       <c r="I401">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J401" t="s">
         <v>30</v>
@@ -16853,7 +16857,7 @@
         <v>3</v>
       </c>
       <c r="I404">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J404" t="s">
         <v>98</v>
@@ -16923,7 +16927,7 @@
         <v>3</v>
       </c>
       <c r="I406">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J406" t="s">
         <v>98</v>
@@ -16958,7 +16962,7 @@
         <v>3</v>
       </c>
       <c r="I407">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J407" t="s">
         <v>25</v>
@@ -16993,7 +16997,7 @@
         <v>3</v>
       </c>
       <c r="I408">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J408" t="s">
         <v>115</v>
@@ -17238,7 +17242,7 @@
         <v>3</v>
       </c>
       <c r="I415">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J415" t="s">
         <v>30</v>
@@ -17378,7 +17382,7 @@
         <v>3</v>
       </c>
       <c r="I419">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J419" t="s">
         <v>415</v>
@@ -17413,7 +17417,7 @@
         <v>3</v>
       </c>
       <c r="I420">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J420" t="s">
         <v>535</v>
@@ -17483,7 +17487,7 @@
         <v>7</v>
       </c>
       <c r="I422">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J422" t="s">
         <v>538</v>
@@ -17763,7 +17767,7 @@
         <v>3</v>
       </c>
       <c r="I430">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J430" t="s">
         <v>125</v>
@@ -17833,7 +17837,7 @@
         <v>3</v>
       </c>
       <c r="I432">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J432" t="s">
         <v>25</v>
@@ -18008,7 +18012,7 @@
         <v>3</v>
       </c>
       <c r="I437">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J437" t="s">
         <v>115</v>
@@ -18043,7 +18047,7 @@
         <v>3</v>
       </c>
       <c r="I438">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J438" t="s">
         <v>25</v>
@@ -18078,7 +18082,7 @@
         <v>3</v>
       </c>
       <c r="I439">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J439" t="s">
         <v>213</v>
@@ -18113,7 +18117,7 @@
         <v>3</v>
       </c>
       <c r="I440">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J440" t="s">
         <v>43</v>
@@ -18148,7 +18152,7 @@
         <v>3</v>
       </c>
       <c r="I441">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J441" t="s">
         <v>136</v>
@@ -18323,7 +18327,7 @@
         <v>7</v>
       </c>
       <c r="I446">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J446" t="s">
         <v>25</v>
@@ -18358,7 +18362,7 @@
         <v>3</v>
       </c>
       <c r="I447">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J447" t="s">
         <v>108</v>
@@ -18428,7 +18432,7 @@
         <v>3</v>
       </c>
       <c r="I449">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J449" t="s">
         <v>30</v>
@@ -18498,7 +18502,7 @@
         <v>3</v>
       </c>
       <c r="I451">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J451" t="s">
         <v>98</v>
@@ -18568,7 +18572,7 @@
         <v>3</v>
       </c>
       <c r="I453">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J453" t="s">
         <v>198</v>
@@ -18708,7 +18712,7 @@
         <v>3</v>
       </c>
       <c r="I457">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J457" t="s">
         <v>30</v>
@@ -18918,7 +18922,7 @@
         <v>3</v>
       </c>
       <c r="I463">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J463" t="s">
         <v>552</v>
@@ -19023,7 +19027,7 @@
         <v>3</v>
       </c>
       <c r="I466">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J466" t="s">
         <v>587</v>
@@ -19058,7 +19062,7 @@
         <v>3</v>
       </c>
       <c r="I467">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J467" t="s">
         <v>64</v>
@@ -19093,7 +19097,7 @@
         <v>7</v>
       </c>
       <c r="I468">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J468" t="s">
         <v>590</v>
@@ -19163,7 +19167,7 @@
         <v>3</v>
       </c>
       <c r="I470">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J470" t="s">
         <v>64</v>
@@ -19268,7 +19272,7 @@
         <v>3</v>
       </c>
       <c r="I473">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J473" t="s">
         <v>342</v>
@@ -19373,7 +19377,7 @@
         <v>3</v>
       </c>
       <c r="I476">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J476" t="s">
         <v>108</v>
@@ -19443,7 +19447,7 @@
         <v>3</v>
       </c>
       <c r="I478">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J478" t="s">
         <v>30</v>
@@ -19513,7 +19517,7 @@
         <v>3</v>
       </c>
       <c r="I480">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J480" t="s">
         <v>30</v>
@@ -19618,7 +19622,7 @@
         <v>3</v>
       </c>
       <c r="I483">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J483" t="s">
         <v>30</v>
@@ -19653,7 +19657,7 @@
         <v>3</v>
       </c>
       <c r="I484">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J484" t="s">
         <v>146</v>
@@ -19688,7 +19692,7 @@
         <v>3</v>
       </c>
       <c r="I485">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J485" t="s">
         <v>30</v>
@@ -19723,7 +19727,7 @@
         <v>3</v>
       </c>
       <c r="I486">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J486" t="s">
         <v>146</v>
@@ -19968,7 +19972,7 @@
         <v>3</v>
       </c>
       <c r="I493">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J493" t="s">
         <v>16</v>
@@ -20003,7 +20007,7 @@
         <v>3</v>
       </c>
       <c r="I494">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J494" t="s">
         <v>16</v>
@@ -20038,7 +20042,7 @@
         <v>3</v>
       </c>
       <c r="I495">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J495" t="s">
         <v>25</v>
@@ -20073,7 +20077,7 @@
         <v>3</v>
       </c>
       <c r="I496">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J496" t="s">
         <v>64</v>
@@ -20108,7 +20112,7 @@
         <v>3</v>
       </c>
       <c r="I497">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J497" t="s">
         <v>621</v>
@@ -20213,7 +20217,7 @@
         <v>3</v>
       </c>
       <c r="I500">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J500" t="s">
         <v>25</v>
@@ -20318,7 +20322,7 @@
         <v>3</v>
       </c>
       <c r="I503">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J503" t="s">
         <v>326</v>
@@ -20353,7 +20357,7 @@
         <v>3</v>
       </c>
       <c r="I504">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J504" t="s">
         <v>629</v>
@@ -20493,7 +20497,7 @@
         <v>3</v>
       </c>
       <c r="I508">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J508" t="s">
         <v>634</v>
@@ -20598,7 +20602,7 @@
         <v>3</v>
       </c>
       <c r="I511">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J511" t="s">
         <v>16</v>
@@ -20633,7 +20637,7 @@
         <v>3</v>
       </c>
       <c r="I512">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J512" t="s">
         <v>639</v>
@@ -20773,7 +20777,7 @@
         <v>3</v>
       </c>
       <c r="I516">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J516" t="s">
         <v>16</v>
@@ -20983,7 +20987,7 @@
         <v>7</v>
       </c>
       <c r="I522">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J522" t="s">
         <v>25</v>
@@ -21018,7 +21022,7 @@
         <v>3</v>
       </c>
       <c r="I523">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J523" t="s">
         <v>30</v>
@@ -21088,7 +21092,7 @@
         <v>3</v>
       </c>
       <c r="I525">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J525" t="s">
         <v>654</v>
@@ -21123,7 +21127,7 @@
         <v>3</v>
       </c>
       <c r="I526">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J526" t="s">
         <v>25</v>
@@ -21193,7 +21197,7 @@
         <v>3</v>
       </c>
       <c r="I528">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J528" t="s">
         <v>658</v>
@@ -21228,7 +21232,7 @@
         <v>3</v>
       </c>
       <c r="I529">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J529" t="s">
         <v>30</v>
@@ -21333,7 +21337,7 @@
         <v>3</v>
       </c>
       <c r="I532">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J532" t="s">
         <v>64</v>
@@ -21368,7 +21372,7 @@
         <v>3</v>
       </c>
       <c r="I533">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J533" t="s">
         <v>25</v>
@@ -21613,7 +21617,7 @@
         <v>3</v>
       </c>
       <c r="I540">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J540" t="s">
         <v>246</v>
@@ -21648,7 +21652,7 @@
         <v>3</v>
       </c>
       <c r="I541">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J541" t="s">
         <v>673</v>
@@ -21763,6 +21767,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M544">
+    <sortCondition ref="A131:A544"/>
+  </sortState>
   <conditionalFormatting sqref="E45:E544">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThanOrEqual">
       <formula>242</formula>

</xml_diff>